<commit_message>
Self checklist: fill author, reviewer and date
</commit_message>
<xml_diff>
--- a/docs/checklist/셀프_체크리스트.xlsx
+++ b/docs/checklist/셀프_체크리스트.xlsx
@@ -917,7 +917,11 @@
           <t>앱 작성자</t>
         </is>
       </c>
-      <c r="C4" s="33" t="n"/>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>광주_2반_김병관</t>
+        </is>
+      </c>
       <c r="D4" s="34" t="n"/>
       <c r="E4" s="35" t="n"/>
       <c r="F4" s="39" t="n"/>
@@ -929,7 +933,11 @@
           <t>점검자</t>
         </is>
       </c>
-      <c r="C5" s="33" t="n"/>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>광주_2반_김병관</t>
+        </is>
+      </c>
       <c r="D5" s="34" t="n"/>
       <c r="E5" s="35" t="n"/>
       <c r="F5" s="39" t="n"/>

</xml_diff>